<commit_message>
CG0277 complete - all test cases validated
</commit_message>
<xml_diff>
--- a/rules/CORE-000469/negative/01/data/unit-test-coreid-CG0277-negative 1.xlsx
+++ b/rules/CORE-000469/negative/01/data/unit-test-coreid-CG0277-negative 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QF\CORE\core-contributor\rules\CORE-000469\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84854509-3208-4CF3-BA46-438D2BA92354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71418AD3-951B-4357-85E3-FD6D18686157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="211">
   <si>
     <t>Product</t>
   </si>
@@ -629,6 +629,42 @@
   </si>
   <si>
     <t>C49666</t>
+  </si>
+  <si>
+    <t>ts.xpt</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Record</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TSGRPID</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TSPARMCD</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>TSVAL</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>INTMODEL</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>STYPE</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>INTERVENTIONAL</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>$STYPE_INTERVENTIONAL</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -712,7 +748,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -728,10 +764,7 @@
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1088,8 +1121,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="6" max="6" width="20.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1109,6 +1147,137 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D2">
+        <v>22</v>
+      </c>
+      <c r="E2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D4">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5">
+        <v>46</v>
+      </c>
+      <c r="E5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6">
+        <v>46</v>
+      </c>
+      <c r="E6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>202</v>
+      </c>
+      <c r="C7" t="s">
+        <v>203</v>
+      </c>
+      <c r="D7">
+        <v>46</v>
+      </c>
+      <c r="E7" t="s">
+        <v>206</v>
+      </c>
+      <c r="F7" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" t="s">
+        <v>203</v>
+      </c>
+      <c r="D8">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s">
+        <v>210</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1695,32 +1864,32 @@
         <v>97</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="8" customFormat="1" ht="43.2" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" s="7">
-        <v>1</v>
-      </c>
-      <c r="D22" s="7"/>
+    <row r="22" spans="1:11" ht="43.2" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="5">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6"/>
       <c r="E22" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="5" t="s">
         <v>99</v>
       </c>
       <c r="G22" s="6"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7" t="s">
+      <c r="H22" s="5"/>
+      <c r="I22" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="J22" s="7" t="s">
+      <c r="J22" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="K22" s="5" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2272,16 +2441,17 @@
       <c r="C46" s="5" t="s">
         <v>121</v>
       </c>
+      <c r="D46" s="7"/>
       <c r="E46" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="F46" s="6" t="s">
+      <c r="F46" s="5" t="s">
         <v>171</v>
       </c>
       <c r="G46" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="H46" s="6"/>
+      <c r="H46" s="5"/>
       <c r="I46" s="5" t="s">
         <v>173</v>
       </c>

</xml_diff>